<commit_message>
Changed main.py to task_1.py to better reflect what's being done.
</commit_message>
<xml_diff>
--- a/data/raw/task1_raw.xlsx
+++ b/data/raw/task1_raw.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eckspur\Documents\!UNIVERSITY\HIT140 (Foundations of Data Science)\FIFA-2026-PROJECT\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD96034F-83C7-448C-8ED8-8988F00EB91F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9F12AB1-D2F8-424E-A1E3-82FBDEEC6948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -673,7 +673,7 @@
         <v>5</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">

</xml_diff>